<commit_message>
Enhance DD modules with detailed function specs and DoD
Co-authored-by: nguyenpr9 <nguyenpr9@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Detail Design v2.xlsx
+++ b/Detail Design v2.xlsx
@@ -18,31 +18,33 @@
     <sheet name="History" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Overview" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Modules" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="DashboardCatalog" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="DashboardLayoutSpec" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="KPI" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="DataModel" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="ModelRelationships" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="SourceMapping" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="DAXLogic" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="BusinessRules" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="RLS" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Module_Function_Spec_v2" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="DashboardCatalog" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="DashboardLayoutSpec" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="KPI" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="DataModel" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="ModelRelationships" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="SourceMapping" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="DAXLogic" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="BusinessRules" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="RLS" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_Reading_Path_v2'!$A$6:$G$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_Reading_Path_v2'!$A$6:$G$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Header'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'History'!$A$1:$D$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Overview'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Modules'!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'DashboardCatalog'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'DashboardLayoutSpec'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'KPI'!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'DataModel'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'ModelRelationships'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'SourceMapping'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'DAXLogic'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'BusinessRules'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'RLS'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Modules'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Module_Function_Spec_v2'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'DashboardCatalog'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'DashboardLayoutSpec'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'KPI'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'DataModel'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'ModelRelationships'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'SourceMapping'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'DAXLogic'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'BusinessRules'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'RLS'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -51,7 +53,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,6 +89,7 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
+    <font/>
   </fonts>
   <fills count="12">
     <fill>
@@ -156,7 +159,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -271,12 +274,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -371,6 +399,19 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1139,7 +1180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G26"/>
+  <dimension ref="B2:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1263,11 +1304,11 @@
           <t>Quick Links - Bắt đầu đọc từ đây</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
-      <c r="F17" s="7" t="n"/>
-      <c r="G17" s="7" t="n"/>
+      <c r="C17" s="38" t="n"/>
+      <c r="D17" s="38" t="n"/>
+      <c r="E17" s="38" t="n"/>
+      <c r="F17" s="38" t="n"/>
+      <c r="G17" s="39" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="36" t="inlineStr">
@@ -1406,10 +1447,40 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>NEW IN v2.2 - Module detail path</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="n"/>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="12" t="n"/>
+      <c r="F28" s="12" t="n"/>
+      <c r="G28" s="12" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="40" t="inlineStr">
+        <is>
+          <t>Bước mới cần đọc sau Modules:</t>
+        </is>
+      </c>
+      <c r="C29" s="41" t="inlineStr">
+        <is>
+          <t>Module_Function_Spec_v2</t>
+        </is>
+      </c>
+      <c r="D29" s="42" t="inlineStr">
+        <is>
+          <t>Mô tả chi tiết từng module cần làm gì ở mức implement</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="B5:D10"/>
     <mergeCell ref="B2:G3"/>
+    <mergeCell ref="B28:G28"/>
     <mergeCell ref="E5:G10"/>
     <mergeCell ref="B17:G17"/>
     <mergeCell ref="B12:G15"/>
@@ -1423,6 +1494,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1434,7 +1506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1442,7 +1514,7 @@
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1540,555 +1612,558 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" s="43" t="n"/>
+      <c r="B9" s="43" t="n"/>
+      <c r="C9" s="43" t="n"/>
+      <c r="D9" s="43" t="n"/>
+      <c r="E9" s="43" t="n"/>
+      <c r="F9" s="43" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="43" t="n"/>
+      <c r="B10" s="43" t="n"/>
+      <c r="C10" s="43" t="n"/>
+      <c r="D10" s="43" t="n"/>
+      <c r="E10" s="43" t="n"/>
+      <c r="F10" s="43" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="43" t="n"/>
+      <c r="B11" s="44" t="n"/>
+      <c r="C11" s="43" t="n"/>
+      <c r="D11" s="43" t="n"/>
+      <c r="E11" s="43" t="n"/>
+      <c r="F11" s="43" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="43" t="n"/>
+      <c r="B12" s="44" t="n"/>
+      <c r="C12" s="43" t="n"/>
+      <c r="D12" s="43" t="n"/>
+      <c r="E12" s="43" t="n"/>
+      <c r="F12" s="43" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="43" t="n"/>
+      <c r="B13" s="44" t="n"/>
+      <c r="C13" s="43" t="n"/>
+      <c r="D13" s="43" t="n"/>
+      <c r="E13" s="43" t="n"/>
+      <c r="F13" s="43" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="43" t="n"/>
+      <c r="B14" s="44" t="n"/>
+      <c r="C14" s="43" t="n"/>
+      <c r="D14" s="43" t="n"/>
+      <c r="E14" s="43" t="n"/>
+      <c r="F14" s="43" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="43" t="n"/>
+      <c r="B15" s="44" t="n"/>
+      <c r="C15" s="43" t="n"/>
+      <c r="D15" s="43" t="n"/>
+      <c r="E15" s="43" t="n"/>
+      <c r="F15" s="43" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="43" t="n"/>
+      <c r="B16" s="44" t="n"/>
+      <c r="C16" s="43" t="n"/>
+      <c r="D16" s="43" t="n"/>
+      <c r="E16" s="43" t="n"/>
+      <c r="F16" s="43" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="43" t="n"/>
+      <c r="B17" s="44" t="n"/>
+      <c r="C17" s="43" t="n"/>
+      <c r="D17" s="43" t="n"/>
+      <c r="E17" s="43" t="n"/>
+      <c r="F17" s="43" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="43" t="n"/>
+      <c r="B18" s="44" t="n"/>
+      <c r="C18" s="43" t="n"/>
+      <c r="D18" s="43" t="n"/>
+      <c r="E18" s="43" t="n"/>
+      <c r="F18" s="43" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="43" t="n"/>
+      <c r="B19" s="44" t="n"/>
+      <c r="C19" s="43" t="n"/>
+      <c r="D19" s="43" t="n"/>
+      <c r="E19" s="43" t="n"/>
+      <c r="F19" s="43" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="43" t="n"/>
+      <c r="B20" s="44" t="n"/>
+      <c r="C20" s="43" t="n"/>
+      <c r="D20" s="43" t="n"/>
+      <c r="E20" s="43" t="n"/>
+      <c r="F20" s="43" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="43" t="n"/>
+      <c r="B21" s="44" t="n"/>
+      <c r="C21" s="43" t="n"/>
+      <c r="D21" s="43" t="n"/>
+      <c r="E21" s="43" t="n"/>
+      <c r="F21" s="43" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="43" t="n"/>
+      <c r="B22" s="44" t="n"/>
+      <c r="C22" s="43" t="n"/>
+      <c r="D22" s="43" t="n"/>
+      <c r="E22" s="43" t="n"/>
+      <c r="F22" s="43" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="43" t="n"/>
+      <c r="B23" s="44" t="n"/>
+      <c r="C23" s="43" t="n"/>
+      <c r="D23" s="43" t="n"/>
+      <c r="E23" s="43" t="n"/>
+      <c r="F23" s="43" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="43" t="n"/>
+      <c r="B24" s="44" t="n"/>
+      <c r="C24" s="43" t="n"/>
+      <c r="D24" s="43" t="n"/>
+      <c r="E24" s="43" t="n"/>
+      <c r="F24" s="43" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="43" t="n"/>
+      <c r="B25" s="44" t="n"/>
+      <c r="C25" s="43" t="n"/>
+      <c r="D25" s="43" t="n"/>
+      <c r="E25" s="43" t="n"/>
+      <c r="F25" s="43" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="43" t="n"/>
+      <c r="B26" s="44" t="n"/>
+      <c r="C26" s="43" t="n"/>
+      <c r="D26" s="43" t="n"/>
+      <c r="E26" s="43" t="n"/>
+      <c r="F26" s="43" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="43" t="n"/>
+      <c r="B27" s="44" t="n"/>
+      <c r="C27" s="43" t="n"/>
+      <c r="D27" s="43" t="n"/>
+      <c r="E27" s="43" t="n"/>
+      <c r="F27" s="43" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>NAVIGATION FROM OVERVIEW</t>
         </is>
       </c>
-      <c r="B9" s="1" t="n"/>
-      <c r="C9" s="1" t="n"/>
-      <c r="D9" s="1" t="n"/>
-      <c r="E9" s="1" t="n"/>
-      <c r="F9" s="1" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="B29" s="1" t="n"/>
+      <c r="C29" s="1" t="n"/>
+      <c r="D29" s="1" t="n"/>
+      <c r="E29" s="1" t="n"/>
+      <c r="F29" s="1" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Đi tới sheet</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>Đọc để làm gì</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E30" s="12" t="inlineStr">
         <is>
           <t>Output</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F30" s="12" t="inlineStr">
         <is>
           <t>Ai nên đọc</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="24" t="n">
+    <row r="31">
+      <c r="A31" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="B11" s="37" t="inlineStr">
-        <is>
-          <t>00_ReadMe_Visual</t>
-        </is>
-      </c>
-      <c r="C11" s="23" t="inlineStr">
-        <is>
-          <t>Nắm roadmap đọc tài liệu detail</t>
-        </is>
-      </c>
-      <c r="D11" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E11" s="23" t="inlineStr">
-        <is>
-          <t>ERD_Star_Visual_v2</t>
-        </is>
-      </c>
-      <c r="F11" s="23" t="inlineStr">
+      <c r="B31" s="37" t="inlineStr">
+        <is>
+          <t>Modules</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="inlineStr">
+        <is>
+          <t>Nắm phạm vi từng module</t>
+        </is>
+      </c>
+      <c r="D31" s="23" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="E31" s="23" t="inlineStr">
+        <is>
+          <t>Module_Function_Spec_v2</t>
+        </is>
+      </c>
+      <c r="F31" s="23" t="inlineStr">
+        <is>
+          <t>PMO + Business</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="B32" s="37" t="inlineStr">
+        <is>
+          <t>Module_Function_Spec_v2</t>
+        </is>
+      </c>
+      <c r="C32" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu chi tiết module cần làm gì ở mức chức năng</t>
+        </is>
+      </c>
+      <c r="D32" s="23" t="inlineStr">
+        <is>
+          <t>Modules</t>
+        </is>
+      </c>
+      <c r="E32" s="23" t="inlineStr">
+        <is>
+          <t>DashboardCatalog</t>
+        </is>
+      </c>
+      <c r="F32" s="23" t="inlineStr">
+        <is>
+          <t>BA + Dev Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="B33" s="37" t="inlineStr">
+        <is>
+          <t>DashboardCatalog</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu dashboard mục tiêu</t>
+        </is>
+      </c>
+      <c r="D33" s="23" t="inlineStr">
+        <is>
+          <t>Function spec</t>
+        </is>
+      </c>
+      <c r="E33" s="23" t="inlineStr">
+        <is>
+          <t>DashboardLayoutSpec</t>
+        </is>
+      </c>
+      <c r="F33" s="23" t="inlineStr">
+        <is>
+          <t>Report Designer</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="B34" s="37" t="inlineStr">
+        <is>
+          <t>DashboardLayoutSpec</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="inlineStr">
+        <is>
+          <t>Chốt visual-level design</t>
+        </is>
+      </c>
+      <c r="D34" s="23" t="inlineStr">
+        <is>
+          <t>DashboardCatalog</t>
+        </is>
+      </c>
+      <c r="E34" s="23" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="F34" s="23" t="inlineStr">
+        <is>
+          <t>Power BI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="B35" s="37" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="C35" s="23" t="inlineStr">
+        <is>
+          <t>Chốt định nghĩa đo lường</t>
+        </is>
+      </c>
+      <c r="D35" s="23" t="inlineStr">
+        <is>
+          <t>Layout spec</t>
+        </is>
+      </c>
+      <c r="E35" s="23" t="inlineStr">
+        <is>
+          <t>Traceability_Matrix_v2</t>
+        </is>
+      </c>
+      <c r="F35" s="23" t="inlineStr">
+        <is>
+          <t>Business + QA</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="B36" s="37" t="inlineStr">
+        <is>
+          <t>Traceability_Matrix_v2</t>
+        </is>
+      </c>
+      <c r="C36" s="23" t="inlineStr">
+        <is>
+          <t>Trace KPI sang DAX/source/test</t>
+        </is>
+      </c>
+      <c r="D36" s="23" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="E36" s="23" t="inlineStr">
+        <is>
+          <t>DataModel</t>
+        </is>
+      </c>
+      <c r="F36" s="23" t="inlineStr">
+        <is>
+          <t>Dev + QA</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="B37" s="37" t="inlineStr">
+        <is>
+          <t>DataModel</t>
+        </is>
+      </c>
+      <c r="C37" s="23" t="inlineStr">
+        <is>
+          <t>Chốt field-level model</t>
+        </is>
+      </c>
+      <c r="D37" s="23" t="inlineStr">
+        <is>
+          <t>Traceability</t>
+        </is>
+      </c>
+      <c r="E37" s="23" t="inlineStr">
+        <is>
+          <t>SourceMapping</t>
+        </is>
+      </c>
+      <c r="F37" s="23" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="B38" s="37" t="inlineStr">
+        <is>
+          <t>SourceMapping</t>
+        </is>
+      </c>
+      <c r="C38" s="23" t="inlineStr">
+        <is>
+          <t>Chốt transform source -&gt; semantic</t>
+        </is>
+      </c>
+      <c r="D38" s="23" t="inlineStr">
+        <is>
+          <t>DataModel</t>
+        </is>
+      </c>
+      <c r="E38" s="23" t="inlineStr">
+        <is>
+          <t>DAXLogic</t>
+        </is>
+      </c>
+      <c r="F38" s="23" t="inlineStr">
+        <is>
+          <t>ETL Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="B39" s="37" t="inlineStr">
+        <is>
+          <t>DAXLogic</t>
+        </is>
+      </c>
+      <c r="C39" s="23" t="inlineStr">
+        <is>
+          <t>Chốt công thức implement</t>
+        </is>
+      </c>
+      <c r="D39" s="23" t="inlineStr">
+        <is>
+          <t>Mapping</t>
+        </is>
+      </c>
+      <c r="E39" s="23" t="inlineStr">
+        <is>
+          <t>BusinessRules</t>
+        </is>
+      </c>
+      <c r="F39" s="23" t="inlineStr">
+        <is>
+          <t>Power BI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="B40" s="37" t="inlineStr">
+        <is>
+          <t>BusinessRules</t>
+        </is>
+      </c>
+      <c r="C40" s="23" t="inlineStr">
+        <is>
+          <t>Chốt rule nghiệp vụ/ngoại lệ</t>
+        </is>
+      </c>
+      <c r="D40" s="23" t="inlineStr">
+        <is>
+          <t>DAX</t>
+        </is>
+      </c>
+      <c r="E40" s="23" t="inlineStr">
+        <is>
+          <t>RLS</t>
+        </is>
+      </c>
+      <c r="F40" s="23" t="inlineStr">
+        <is>
+          <t>Business + QA</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="24" t="n">
+        <v>11</v>
+      </c>
+      <c r="B41" s="37" t="inlineStr">
+        <is>
+          <t>RLS</t>
+        </is>
+      </c>
+      <c r="C41" s="23" t="inlineStr">
+        <is>
+          <t>Chốt phân quyền dữ liệu</t>
+        </is>
+      </c>
+      <c r="D41" s="23" t="inlineStr">
+        <is>
+          <t>BusinessRules</t>
+        </is>
+      </c>
+      <c r="E41" s="23" t="inlineStr">
+        <is>
+          <t>Refresh_Monitor_v2</t>
+        </is>
+      </c>
+      <c r="F41" s="23" t="inlineStr">
+        <is>
+          <t>Security + Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="B42" s="37" t="inlineStr">
+        <is>
+          <t>Refresh_Monitor_v2</t>
+        </is>
+      </c>
+      <c r="C42" s="23" t="inlineStr">
+        <is>
+          <t>Theo dõi vận hành sau triển khai</t>
+        </is>
+      </c>
+      <c r="D42" s="23" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="24" t="n">
-        <v>2</v>
-      </c>
-      <c r="B12" s="37" t="inlineStr">
-        <is>
-          <t>ERD_Star_Visual_v2</t>
-        </is>
-      </c>
-      <c r="C12" s="23" t="inlineStr">
-        <is>
-          <t>Hiểu cấu trúc star schema trực quan</t>
-        </is>
-      </c>
-      <c r="D12" s="23" t="inlineStr">
-        <is>
-          <t>ReadMe</t>
-        </is>
-      </c>
-      <c r="E12" s="23" t="inlineStr">
-        <is>
-          <t>ETL_Swimlane_v2</t>
-        </is>
-      </c>
-      <c r="F12" s="23" t="inlineStr">
-        <is>
-          <t>Data + BI Dev</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="B13" s="37" t="inlineStr">
-        <is>
-          <t>ETL_Swimlane_v2</t>
-        </is>
-      </c>
-      <c r="C13" s="23" t="inlineStr">
-        <is>
-          <t>Hiểu trình tự ETL và các gate kiểm soát</t>
-        </is>
-      </c>
-      <c r="D13" s="23" t="inlineStr">
-        <is>
-          <t>ERD</t>
-        </is>
-      </c>
-      <c r="E13" s="23" t="inlineStr">
-        <is>
-          <t>Overview</t>
-        </is>
-      </c>
-      <c r="F13" s="23" t="inlineStr">
-        <is>
-          <t>Data Engineer</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="24" t="n">
-        <v>4</v>
-      </c>
-      <c r="B14" s="37" t="inlineStr">
-        <is>
-          <t>Overview</t>
-        </is>
-      </c>
-      <c r="C14" s="23" t="inlineStr">
-        <is>
-          <t>Hiểu SLA, tầng dữ liệu, giả định triển khai</t>
-        </is>
-      </c>
-      <c r="D14" s="23" t="inlineStr">
-        <is>
-          <t>ETL Flow</t>
-        </is>
-      </c>
-      <c r="E14" s="23" t="inlineStr">
-        <is>
-          <t>Modules</t>
-        </is>
-      </c>
-      <c r="F14" s="23" t="inlineStr">
-        <is>
-          <t>Architect + PM</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="24" t="n">
-        <v>5</v>
-      </c>
-      <c r="B15" s="37" t="inlineStr">
-        <is>
-          <t>Modules</t>
-        </is>
-      </c>
-      <c r="C15" s="23" t="inlineStr">
-        <is>
-          <t>Hiểu phạm vi từng subject area</t>
-        </is>
-      </c>
-      <c r="D15" s="23" t="inlineStr">
-        <is>
-          <t>Overview</t>
-        </is>
-      </c>
-      <c r="E15" s="23" t="inlineStr">
-        <is>
-          <t>DashboardCatalog</t>
-        </is>
-      </c>
-      <c r="F15" s="23" t="inlineStr">
-        <is>
-          <t>Business</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="24" t="n">
-        <v>6</v>
-      </c>
-      <c r="B16" s="37" t="inlineStr">
-        <is>
-          <t>DashboardCatalog</t>
-        </is>
-      </c>
-      <c r="C16" s="23" t="inlineStr">
-        <is>
-          <t>Hiểu mục tiêu từng dashboard</t>
-        </is>
-      </c>
-      <c r="D16" s="23" t="inlineStr">
-        <is>
-          <t>Modules</t>
-        </is>
-      </c>
-      <c r="E16" s="23" t="inlineStr">
-        <is>
-          <t>DashboardLayoutSpec</t>
-        </is>
-      </c>
-      <c r="F16" s="23" t="inlineStr">
-        <is>
-          <t>Report Designer</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="24" t="n">
-        <v>7</v>
-      </c>
-      <c r="B17" s="37" t="inlineStr">
-        <is>
-          <t>DashboardLayoutSpec</t>
-        </is>
-      </c>
-      <c r="C17" s="23" t="inlineStr">
-        <is>
-          <t>Hiểu vị trí visual + field binding</t>
-        </is>
-      </c>
-      <c r="D17" s="23" t="inlineStr">
-        <is>
-          <t>DashboardCatalog</t>
-        </is>
-      </c>
-      <c r="E17" s="23" t="inlineStr">
-        <is>
-          <t>KPI</t>
-        </is>
-      </c>
-      <c r="F17" s="23" t="inlineStr">
-        <is>
-          <t>Power BI Dev</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="24" t="n">
-        <v>8</v>
-      </c>
-      <c r="B18" s="37" t="inlineStr">
-        <is>
-          <t>KPI</t>
-        </is>
-      </c>
-      <c r="C18" s="23" t="inlineStr">
-        <is>
-          <t>Hiểu business definition + ngưỡng KPI</t>
-        </is>
-      </c>
-      <c r="D18" s="23" t="inlineStr">
-        <is>
-          <t>Dashboard Spec</t>
-        </is>
-      </c>
-      <c r="E18" s="23" t="inlineStr">
-        <is>
-          <t>Traceability_Matrix_v2</t>
-        </is>
-      </c>
-      <c r="F18" s="23" t="inlineStr">
-        <is>
-          <t>Business + QA</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="24" t="n">
-        <v>9</v>
-      </c>
-      <c r="B19" s="37" t="inlineStr">
-        <is>
-          <t>Traceability_Matrix_v2</t>
-        </is>
-      </c>
-      <c r="C19" s="23" t="inlineStr">
-        <is>
-          <t>Trace KPI -&gt; DAX -&gt; Source -&gt; Test</t>
-        </is>
-      </c>
-      <c r="D19" s="23" t="inlineStr">
-        <is>
-          <t>KPI</t>
-        </is>
-      </c>
-      <c r="E19" s="23" t="inlineStr">
-        <is>
-          <t>DataModel</t>
-        </is>
-      </c>
-      <c r="F19" s="23" t="inlineStr">
-        <is>
-          <t>Dev + QA</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="24" t="n">
-        <v>10</v>
-      </c>
-      <c r="B20" s="37" t="inlineStr">
-        <is>
-          <t>DataModel</t>
-        </is>
-      </c>
-      <c r="C20" s="23" t="inlineStr">
-        <is>
-          <t>Chi tiết field-level cho Fact/Dim</t>
-        </is>
-      </c>
-      <c r="D20" s="23" t="inlineStr">
-        <is>
-          <t>Traceability</t>
-        </is>
-      </c>
-      <c r="E20" s="23" t="inlineStr">
-        <is>
-          <t>ModelRelationships</t>
-        </is>
-      </c>
-      <c r="F20" s="23" t="inlineStr">
-        <is>
-          <t>Data Modeler</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="24" t="n">
-        <v>11</v>
-      </c>
-      <c r="B21" s="37" t="inlineStr">
-        <is>
-          <t>ModelRelationships</t>
-        </is>
-      </c>
-      <c r="C21" s="23" t="inlineStr">
-        <is>
-          <t>Hiểu cardinality/filter direction</t>
-        </is>
-      </c>
-      <c r="D21" s="23" t="inlineStr">
-        <is>
-          <t>DataModel</t>
-        </is>
-      </c>
-      <c r="E21" s="23" t="inlineStr">
-        <is>
-          <t>SourceMapping</t>
-        </is>
-      </c>
-      <c r="F21" s="23" t="inlineStr">
-        <is>
-          <t>Power BI Dev</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="24" t="n">
-        <v>12</v>
-      </c>
-      <c r="B22" s="37" t="inlineStr">
-        <is>
-          <t>SourceMapping</t>
-        </is>
-      </c>
-      <c r="C22" s="23" t="inlineStr">
-        <is>
-          <t>Map source field -&gt; semantic field + transform</t>
-        </is>
-      </c>
-      <c r="D22" s="23" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="E22" s="23" t="inlineStr">
-        <is>
-          <t>DAXLogic</t>
-        </is>
-      </c>
-      <c r="F22" s="23" t="inlineStr">
-        <is>
-          <t>ETL Dev</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="24" t="n">
-        <v>13</v>
-      </c>
-      <c r="B23" s="37" t="inlineStr">
-        <is>
-          <t>DAXLogic</t>
-        </is>
-      </c>
-      <c r="C23" s="23" t="inlineStr">
-        <is>
-          <t>Công thức DAX đầy đủ + test case</t>
-        </is>
-      </c>
-      <c r="D23" s="23" t="inlineStr">
-        <is>
-          <t>KPI + Mapping</t>
-        </is>
-      </c>
-      <c r="E23" s="23" t="inlineStr">
-        <is>
-          <t>BusinessRules</t>
-        </is>
-      </c>
-      <c r="F23" s="23" t="inlineStr">
-        <is>
-          <t>Power BI Dev</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="24" t="n">
-        <v>14</v>
-      </c>
-      <c r="B24" s="37" t="inlineStr">
-        <is>
-          <t>BusinessRules</t>
-        </is>
-      </c>
-      <c r="C24" s="23" t="inlineStr">
-        <is>
-          <t>Luật nghiệp vụ và ngoại lệ ngành xây dựng</t>
-        </is>
-      </c>
-      <c r="D24" s="23" t="inlineStr">
-        <is>
-          <t>DAX</t>
-        </is>
-      </c>
-      <c r="E24" s="23" t="inlineStr">
-        <is>
-          <t>RLS_Heatmap_v2</t>
-        </is>
-      </c>
-      <c r="F24" s="23" t="inlineStr">
-        <is>
-          <t>Business + QA</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="24" t="n">
-        <v>15</v>
-      </c>
-      <c r="B25" s="37" t="inlineStr">
-        <is>
-          <t>RLS_Heatmap_v2</t>
-        </is>
-      </c>
-      <c r="C25" s="23" t="inlineStr">
-        <is>
-          <t>Nhìn nhanh phạm vi role và access</t>
-        </is>
-      </c>
-      <c r="D25" s="23" t="inlineStr">
-        <is>
-          <t>BusinessRules</t>
-        </is>
-      </c>
-      <c r="E25" s="23" t="inlineStr">
-        <is>
-          <t>RLS</t>
-        </is>
-      </c>
-      <c r="F25" s="23" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="24" t="n">
-        <v>16</v>
-      </c>
-      <c r="B26" s="37" t="inlineStr">
-        <is>
-          <t>RLS</t>
-        </is>
-      </c>
-      <c r="C26" s="23" t="inlineStr">
-        <is>
-          <t>DAX filter role-level cho Power BI Service</t>
-        </is>
-      </c>
-      <c r="D26" s="23" t="inlineStr">
-        <is>
-          <t>RLS Heatmap</t>
-        </is>
-      </c>
-      <c r="E26" s="23" t="inlineStr">
-        <is>
-          <t>Refresh_Monitor_v2</t>
-        </is>
-      </c>
-      <c r="F26" s="23" t="inlineStr">
-        <is>
-          <t>Security + Admin</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="24" t="n">
-        <v>17</v>
-      </c>
-      <c r="B27" s="37" t="inlineStr">
-        <is>
-          <t>Refresh_Monitor_v2</t>
-        </is>
-      </c>
-      <c r="C27" s="23" t="inlineStr">
-        <is>
-          <t>Theo dõi vận hành refresh/DQ sau triển khai</t>
-        </is>
-      </c>
-      <c r="D27" s="23" t="inlineStr">
-        <is>
-          <t>All implementation</t>
-        </is>
-      </c>
-      <c r="E27" s="23" t="inlineStr">
+      <c r="E42" s="23" t="inlineStr">
         <is>
           <t>Runbook</t>
         </is>
       </c>
-      <c r="F27" s="23" t="inlineStr">
+      <c r="F42" s="23" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
@@ -2097,7 +2172,7 @@
   </sheetData>
   <autoFilter ref="A1:B1"/>
   <mergeCells count="1">
-    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A29:F29"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId1"/>
@@ -2117,6 +2192,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2128,18 +2215,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="64" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="61" customWidth="1" min="8" max="8"/>
+    <col width="72" customWidth="1" min="9" max="9"/>
+    <col width="72" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2180,10 +2270,25 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Chức năng chi tiết cần triển khai (Must-Have)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Integration / Dependencies</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Definition of Done (DoD)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Tần suất refresh</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>SLA</t>
         </is>
@@ -2227,10 +2332,29 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
+          <t>1) Theo dõi nhập-xuất-trả theo ngày/công trình/work package
+2) Tính NetQty, OverNormQty ở mức transaction
+3) Drillthrough tới chứng từ nguồn
+4) Cảnh báo overuse theo ngưỡng 5/10%
+5) Phân tích mix vật tư theo nhóm + contractor</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Phụ thuộc BOM approved, DimMaterial chuẩn hóa, mapping WorkPackage; đồng bộ với module tiến độ để kiểm tra mức tiêu hao theo khối lượng thực hiện.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Dashboard hiển thị đúng KPI theo test case TC-KPI-001/002; giao dịch thiếu BOM được tách trạng thái Data Issue; PM drill tới DocNo được.</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
           <t>2 giờ/lần</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Freshness &lt;= 2h</t>
         </is>
@@ -2274,10 +2398,29 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
+          <t>1) So sánh PlannedQty vs ActualCompletedQty theo tuần
+2) Tính DelayDays và phân tầng risk level
+3) Theo dõi milestone critical path
+4) Cảnh báo SPI &lt; 0.95
+5) Drilldown Project -&gt; Phase -&gt; WorkPackage</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Phụ thuộc DimDate, DimWorkPackage và dữ liệu baseline được khóa phiên bản; dùng cùng chuẩn ProjectKey với cost/material để phân tích liên thông.</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Trend line, milestone table, risk matrix khớp dữ liệu nguồn; quy tắc cap tiến độ &lt;=100% hoạt động đúng; delay âm được ép 0.</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
           <t>2 giờ/lần</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Freshness &lt;= 2h</t>
         </is>
@@ -2321,10 +2464,29 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
+          <t>1) Tổng hợp Budget/Actual/Committed theo category
+2) Tính Variance và Variance% theo nhiều cấp
+3) Waterfall phân rã nguyên nhân chênh lệch
+4) Theo dõi ChangeOrder tác động ngân sách
+5) Cảnh báo &gt;5% (vàng), &gt;10% (đỏ)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Phụ thuộc chuẩn CostCategory hierarchy, quy đổi tiền tệ VND và loại bỏ reversal; cần liên kết EV từ module tiến độ để tính CPI.</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>KPI chi phí đối soát với finance ledger sai lệch &lt;=0.5%; matrix drilldown đầy đủ 3 tầng; màu cảnh báo đúng ngưỡng.</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
           <t>2 giờ/lần</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Freshness &lt;= 2h</t>
         </is>
@@ -2368,10 +2530,29 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
+          <t>1) Xếp hạng nhà thầu theo productivity/cost/schedule
+2) Tính On-time delivery theo ETA ±1 ngày
+3) Theo dõi lỗi SLA theo loại vi phạm
+4) Benchmark giữa các nhà thầu cùng loại
+5) Cảnh báo nhà thầu dưới ngưỡng tier B</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Phụ thuộc dữ liệu labor hours, delivery log và mapping contractor-company cho RLS; dùng dữ liệu kết hợp từ material + progress + cost.</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Scorecard tái lập được theo tháng; rule loại bản ghi thiếu labor hour hoạt động đúng; contractor external chỉ thấy dữ liệu own company.</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
           <t>Ngày</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Daily 06:00</t>
         </is>
@@ -2415,22 +2596,1160 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
+          <t>1) Theo dõi accepted qty theo giai đoạn
+2) So sánh thi công thực tế vs nghiệm thu
+3) Theo dõi hồ sơ thanh toán pending/approved/paid
+4) Cảnh báo quá hạn thanh toán theo SLA
+5) Drillthrough tới biên bản nghiệm thu</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Phụ thuộc chứng từ nghiệm thu chuẩn hóa và status workflow thanh toán; cần liên kết với tiến độ để tránh nghiệm thu vượt thực tế.</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Báo cáo thể hiện đúng trạng thái hồ sơ; pending amount tính đúng theo kỳ; drillthrough biên bản/phiếu thanh toán hoạt động.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
           <t>Ngày</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Daily 06:00</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
+  <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="41" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Module ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Function ID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Function Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Mô tả chi tiết cần làm</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Input chính</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Logic xử lý chính</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Output / Visual</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>M01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>M01-F01</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Material Ledger Consolidation</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Hợp nhất phiếu xuất, phiếu trả, điều chỉnh tồn theo ngày và WorkPackage.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>MaterialIssueLine, MaterialReturnLine</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>NetQty = Issued - Return; loại chứng từ cancelled.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Table giao dịch + KPI NetQty</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Số liệu khớp tổng source lệch &lt;=0.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>M01</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>M01-F02</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Overuse Detection</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tính lượng vượt định mức theo BOM version hiệu lực.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>BOMNorm + NetQty</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>OverNormQty = max(NetQty - NormQty,0).</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>KPI Overuse % + Heatmap</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>BI Developer</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Ngưỡng cảnh báo 5/10% hiển thị đúng màu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>M01</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>M01-F03</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Material Mix Analysis</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Phân tích cơ cấu vật tư theo nhóm / dự án / nhà thầu.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>DimMaterial + FactMaterialConsumption</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Tính share theo filter context.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Donut + stacked column</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>BI Analyst</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Top nhóm vật tư đúng theo filter</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>M01</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>M01-F04</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Document Drillthrough</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Drillthrough từ KPI/heatmap xuống chứng từ nguồn.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>SourceDocNo, ProjectKey</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Giữ grain transaction để trace.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Drillthrough page</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>BI Developer</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Click 1 dòng mở đúng chứng từ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>M02</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>M02-F01</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Progress Baseline Comparison</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>So sánh tiến độ baseline vs actual theo tuần.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>ProgressDaily, WorkPackagePlan</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Planned%/Actual% theo BaselineQty.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Line trend planned vs actual</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Planning BI Analyst</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Trend khớp bảng tiến độ nguồn</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>M02</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>M02-F02</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Delay Risk Scoring</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Chấm điểm rủi ro theo DelayDays + SPI.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>DelayDays, SPI</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Risk = High/Medium/Low theo rule BR.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Risk matrix</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>BI Developer</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Rule biên 7/14 ngày đúng</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>M02</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>M02-F03</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Milestone Tracking</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi milestone critical với cảnh báo quá hạn.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Milestone schedule</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>DelayDays = max(0, Forecast-Plan).</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Milestone warning table</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Planning Engineer</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Milestone quá hạn tô màu đỏ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>M02</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>M02-F04</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>WorkPackage Drill Path</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Drill Project -&gt; Phase -&gt; WorkPackage để khoanh vùng chậm.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>DimWorkPackage, FactProgressTracking</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Hierarchy filter context chính xác.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Matrix drilldown</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>BI Developer</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Drill path không mất ngữ cảnh</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>M03</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>M03-F01</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Budget-Actual Consolidation</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Tổng hợp budget, actual, committed theo category và kỳ.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>BudgetBaseline, CostLedger, CommitmentLedger</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Loại reversal, quy đổi VND.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>KPI cards + matrix</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Finance BI Analyst</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Đối soát finance pass &lt;=0.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>M03</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>M03-F02</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Variance Waterfall</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Phân rã nguyên nhân chênh lệch ngân sách.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>FactProjectCost, DimCostCategory</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Variance = Actual - Budget theo driver.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Waterfall chart</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>BI Analyst</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Top driver đúng với matrix</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>M03</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>M03-F03</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Alerting Rules</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Thiết lập cảnh báo vượt 5%/10%.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Budget Variance %</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Rule màu vàng/đỏ theo threshold.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Card + conditional matrix</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>BI Developer</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Màu cảnh báo đúng ngưỡng</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>M03</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>M03-F04</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Change Order Impact</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Phân tích tác động phát sinh lên ngân sách.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>ChangeOrder</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi delta trước/sau CO.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Bar + trend line</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>PMO Analyst</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>CO approved mới được tính</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>M04</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>M04-F01</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Productivity Score</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Tính năng suất theo sản lượng/giờ công.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>ActualCompletedQty, LaborHours</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Productivity = Qty/LaborHours; loại zero hours.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Scorecard KPI</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Contract Manager</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Top/Bottom contractor đúng logic</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>M04</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>M04-F02</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>On-time Delivery SLA</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Đo tỷ lệ giao hàng đúng hạn ETA ±1 ngày.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>DeliveryPerformance</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>On-time count / total count.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>SLA bar chart</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Procurement Analyst</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Tỷ lệ đúng với log giao nhận</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>M04</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>M04-F03</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Benchmark</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>So sánh nhà thầu cùng nhóm công việc.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>DimContractor, KPI scores</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Ranking theo weighted score.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Benchmark matrix</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>BI Analyst</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Ranking ổn định theo kỳ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>M04</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>M04-F04</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>External Access Scope</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Giới hạn nhà thầu chỉ thấy dữ liệu own company.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>SecurityUserProject, CompanyCode</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>RLS filter theo company.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>External contractor view</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Security Admin</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Tài khoản ngoài chỉ thấy dữ liệu hợp lệ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>M05</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>M05-F01</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance Progress Tracking</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi accepted qty theo phase/work package.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>AcceptanceMinutes</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>AcceptedQty tổng hợp theo kỳ.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance trend</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>QS Analyst</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Accepted qty khớp biên bản</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>M05</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>M05-F02</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Construction vs Acceptance Reconcile</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Đối soát thi công thực tế với nghiệm thu.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>FactProgressTracking + Acceptance</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Variance giữa actual completed và accepted.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Variance table</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Site Engineer</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Sai lệch vượt ngưỡng được cảnh báo</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>M05</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>M05-F03</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Billing Workflow Monitor</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi trạng thái pending/approved/paid hồ sơ.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>BillingProgress, PaymentCertificate</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Status lifecycle theo ngày xử lý.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Workflow funnel + table</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Finance Ops</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Pending quá SLA hiển thị đỏ</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>M05</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>M05-F04</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Payment Delay Alert</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Cảnh báo hồ sơ thanh toán quá hạn SLA.</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>DueDate, PaymentDate</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Delay = max(0, PaymentDate-DueDate).</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Delay alert dashboard</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Finance Controller</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Danh sách quá hạn đúng theo source</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2648,7 +3967,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3387,7 +4706,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3836,7 +5155,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6672,7 +7991,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7327,7 +8646,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9793,7 +11112,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10294,452 +11613,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="85" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Rule ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Phân hệ</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Luật nghiệp vụ chi tiết</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Điểm triển khai</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Xử lý ngoại lệ</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Data Owner</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>BR-01</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Mã vật tư phải map MaterialGroup; không map gán UNCLASSIFIED và alert 08:00 mỗi ngày.</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>ETL SQL + Power Query</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Vẫn load nhưng loại khỏi KPI chiến lược.</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>MDM Team</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>BR-02</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>NormQty lấy theo BOM approved mới nhất có EffectiveDate &lt;= ngày giao dịch.</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>ETL SQL</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Không có BOM thì Overuse KPI trả BLANK và log DQ.</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Engineering Control</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>BR-03</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Project</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Chỉ load dự án Status IN ('Active','Closing'); Closed giữ tối đa 24 tháng.</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>ETL SQL</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Audit sâu dùng workspace archive.</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>PMO</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>BR-04</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>ActualAmount loại bút toán reversal/cancelled theo trạng thái chứng từ.</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>ETL SQL</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Reversal đến sau cutoff ghi adjustment kỳ kế tiếp.</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>BR-05</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Quy đổi currency về VND theo tỷ giá cuối tháng; thiếu rate dùng nearest previous.</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Power Query + SQL</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Thiếu rate &gt;7 ngày đánh critical.</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Treasury</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>BR-06</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Progress</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>DelayDays = max(0, ForecastFinishDate - PlannedFinishDate).</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>ETL SQL</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Forecast null dùng RevisedFinishDate.</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Planning Office</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>BR-07</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Progress</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Actual Progress % cap 100% để tránh outlier do baseline cập nhật trễ.</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>DAX</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Record &gt;100% được log để PM xác nhận.</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Planning Office</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>BR-08</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Productivity Index chỉ tính khi LaborHours&gt;0 và ActualCompletedQty&gt;0.</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>DAX</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Record không hợp lệ đưa vào trang Data Quality.</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Contract Management</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>BR-09</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>User chỉ xem dự án mapping trong SecurityUserProject và IsActive=1.</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>RLS DAX</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>User không mapping sẽ không thấy dữ liệu.</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>IT Security</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>BR-10</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Khóa số liệu tháng vào T+3 18:00; sửa sau khóa cần approval ticket.</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Process + SQL</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Lưu audit trail DataCorrectionLog.</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>PMO + Data Governance</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>BR-11</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Executive dashboard chỉ hiển thị Top 15 dự án theo Actual Cost để tối ưu hiệu năng.</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Visual Filter</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Danh sách đầy đủ ở drillthrough.</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>BI Team</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>BR-12</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Quality</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Đối soát KPI semantic vs source hằng ngày; sai lệch cho phép &lt;=0.5%.</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>SQL Validation Job</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Lệch &gt;0.5% thì refresh fail + gửi alert.</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Data Quality Team</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10754,7 +11634,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DETAIL DESIGN - RECOMMENDED READING PATH</t>
+          <t>DETAIL DESIGN - RECOMMENDED READING PATH (UPDATED WITH MODULE FUNCTION SPEC)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -10774,59 +11654,59 @@
       <c r="G2" s="1" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="36" t="inlineStr">
-        <is>
-          <t>Đọc theo thứ tự từ trên xuống. Cột "Liên kết sheet" có hyperlink để nhảy trực tiếp tới sheet tương ứng.</t>
-        </is>
-      </c>
-      <c r="B3" s="36" t="n"/>
-      <c r="C3" s="36" t="n"/>
-      <c r="D3" s="36" t="n"/>
-      <c r="E3" s="36" t="n"/>
-      <c r="F3" s="36" t="n"/>
-      <c r="G3" s="36" t="n"/>
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>Đọc theo thứ tự. Cột "Liên kết sheet" có hyperlink. Bổ sung bước Module_Function_Spec_v2 để dev biết rõ từng module cần làm gì.</t>
+        </is>
+      </c>
+      <c r="B3" s="40" t="n"/>
+      <c r="C3" s="40" t="n"/>
+      <c r="D3" s="40" t="n"/>
+      <c r="E3" s="40" t="n"/>
+      <c r="F3" s="40" t="n"/>
+      <c r="G3" s="40" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="36" t="n"/>
-      <c r="B4" s="36" t="n"/>
-      <c r="C4" s="36" t="n"/>
-      <c r="D4" s="36" t="n"/>
-      <c r="E4" s="36" t="n"/>
-      <c r="F4" s="36" t="n"/>
-      <c r="G4" s="36" t="n"/>
+      <c r="A4" s="40" t="n"/>
+      <c r="B4" s="40" t="n"/>
+      <c r="C4" s="40" t="n"/>
+      <c r="D4" s="40" t="n"/>
+      <c r="E4" s="40" t="n"/>
+      <c r="F4" s="40" t="n"/>
+      <c r="G4" s="40" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Liên kết sheet</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>Mục tiêu đọc</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Input nhận từ</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>Output chuyển tới</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>Persona chính</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>Kết quả kỳ vọng</t>
         </is>
@@ -10913,7 +11793,7 @@
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Hiểu trình tự ETL và các gate kiểm soát</t>
+          <t>Hiểu trình tự ETL và gate kiểm soát</t>
         </is>
       </c>
       <c r="D9" s="23" t="inlineStr">
@@ -10983,7 +11863,7 @@
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>Hiểu phạm vi từng subject area</t>
+          <t>Hiểu phạm vi module và mục tiêu nghiệp vụ</t>
         </is>
       </c>
       <c r="D11" s="23" t="inlineStr">
@@ -10993,17 +11873,17 @@
       </c>
       <c r="E11" s="23" t="inlineStr">
         <is>
-          <t>DashboardCatalog</t>
+          <t>Module_Function_Spec_v2</t>
         </is>
       </c>
       <c r="F11" s="23" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Business + PMO</t>
         </is>
       </c>
       <c r="G11" s="23" t="inlineStr">
         <is>
-          <t>Ưu tiên backlog</t>
+          <t>Chốt scope theo module</t>
         </is>
       </c>
     </row>
@@ -11013,32 +11893,32 @@
       </c>
       <c r="B12" s="37" t="inlineStr">
         <is>
+          <t>Module_Function_Spec_v2</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu chi tiết từng module cần làm gì ở mức chức năng</t>
+        </is>
+      </c>
+      <c r="D12" s="23" t="inlineStr">
+        <is>
+          <t>Modules</t>
+        </is>
+      </c>
+      <c r="E12" s="23" t="inlineStr">
+        <is>
           <t>DashboardCatalog</t>
         </is>
       </c>
-      <c r="C12" s="23" t="inlineStr">
-        <is>
-          <t>Hiểu mục tiêu từng dashboard</t>
-        </is>
-      </c>
-      <c r="D12" s="23" t="inlineStr">
-        <is>
-          <t>Modules</t>
-        </is>
-      </c>
-      <c r="E12" s="23" t="inlineStr">
-        <is>
-          <t>DashboardLayoutSpec</t>
-        </is>
-      </c>
       <c r="F12" s="23" t="inlineStr">
         <is>
-          <t>Report Designer</t>
+          <t>Dev Lead + BA</t>
         </is>
       </c>
       <c r="G12" s="23" t="inlineStr">
         <is>
-          <t>Chốt trang báo cáo</t>
+          <t>Lập backlog implement rõ ràng</t>
         </is>
       </c>
     </row>
@@ -11048,32 +11928,32 @@
       </c>
       <c r="B13" s="37" t="inlineStr">
         <is>
+          <t>DashboardCatalog</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu mục tiêu từng dashboard</t>
+        </is>
+      </c>
+      <c r="D13" s="23" t="inlineStr">
+        <is>
+          <t>Module function spec</t>
+        </is>
+      </c>
+      <c r="E13" s="23" t="inlineStr">
+        <is>
           <t>DashboardLayoutSpec</t>
         </is>
       </c>
-      <c r="C13" s="23" t="inlineStr">
-        <is>
-          <t>Hiểu vị trí visual + field binding</t>
-        </is>
-      </c>
-      <c r="D13" s="23" t="inlineStr">
-        <is>
-          <t>DashboardCatalog</t>
-        </is>
-      </c>
-      <c r="E13" s="23" t="inlineStr">
-        <is>
-          <t>KPI</t>
-        </is>
-      </c>
       <c r="F13" s="23" t="inlineStr">
         <is>
-          <t>Power BI Dev</t>
+          <t>Report Designer</t>
         </is>
       </c>
       <c r="G13" s="23" t="inlineStr">
         <is>
-          <t>Triển khai UI/UX report</t>
+          <t>Chốt trang báo cáo</t>
         </is>
       </c>
     </row>
@@ -11083,32 +11963,32 @@
       </c>
       <c r="B14" s="37" t="inlineStr">
         <is>
+          <t>DashboardLayoutSpec</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu vị trí visual + field binding</t>
+        </is>
+      </c>
+      <c r="D14" s="23" t="inlineStr">
+        <is>
+          <t>DashboardCatalog</t>
+        </is>
+      </c>
+      <c r="E14" s="23" t="inlineStr">
+        <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="C14" s="23" t="inlineStr">
-        <is>
-          <t>Hiểu business definition + ngưỡng KPI</t>
-        </is>
-      </c>
-      <c r="D14" s="23" t="inlineStr">
-        <is>
-          <t>Dashboard Spec</t>
-        </is>
-      </c>
-      <c r="E14" s="23" t="inlineStr">
-        <is>
-          <t>Traceability_Matrix_v2</t>
-        </is>
-      </c>
       <c r="F14" s="23" t="inlineStr">
         <is>
-          <t>Business + QA</t>
+          <t>Power BI Dev</t>
         </is>
       </c>
       <c r="G14" s="23" t="inlineStr">
         <is>
-          <t>Chốt tiêu chí nghiệm thu</t>
+          <t>Triển khai UI/UX report</t>
         </is>
       </c>
     </row>
@@ -11118,32 +11998,32 @@
       </c>
       <c r="B15" s="37" t="inlineStr">
         <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu business definition + ngưỡng KPI</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="inlineStr">
+        <is>
+          <t>Dashboard spec</t>
+        </is>
+      </c>
+      <c r="E15" s="23" t="inlineStr">
+        <is>
           <t>Traceability_Matrix_v2</t>
         </is>
       </c>
-      <c r="C15" s="23" t="inlineStr">
-        <is>
-          <t>Trace KPI -&gt; DAX -&gt; Source -&gt; Test</t>
-        </is>
-      </c>
-      <c r="D15" s="23" t="inlineStr">
-        <is>
-          <t>KPI</t>
-        </is>
-      </c>
-      <c r="E15" s="23" t="inlineStr">
-        <is>
-          <t>DataModel</t>
-        </is>
-      </c>
       <c r="F15" s="23" t="inlineStr">
         <is>
-          <t>Dev + QA</t>
+          <t>Business + QA</t>
         </is>
       </c>
       <c r="G15" s="23" t="inlineStr">
         <is>
-          <t>Không thiếu mapping</t>
+          <t>Chốt tiêu chí nghiệm thu</t>
         </is>
       </c>
     </row>
@@ -11153,32 +12033,32 @@
       </c>
       <c r="B16" s="37" t="inlineStr">
         <is>
+          <t>Traceability_Matrix_v2</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>Trace KPI -&gt; DAX -&gt; Source -&gt; Test</t>
+        </is>
+      </c>
+      <c r="D16" s="23" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="E16" s="23" t="inlineStr">
+        <is>
           <t>DataModel</t>
         </is>
       </c>
-      <c r="C16" s="23" t="inlineStr">
-        <is>
-          <t>Chi tiết field-level cho Fact/Dim</t>
-        </is>
-      </c>
-      <c r="D16" s="23" t="inlineStr">
-        <is>
-          <t>Traceability</t>
-        </is>
-      </c>
-      <c r="E16" s="23" t="inlineStr">
-        <is>
-          <t>ModelRelationships</t>
-        </is>
-      </c>
       <c r="F16" s="23" t="inlineStr">
         <is>
-          <t>Data Modeler</t>
+          <t>Dev + QA</t>
         </is>
       </c>
       <c r="G16" s="23" t="inlineStr">
         <is>
-          <t>Build model chính xác</t>
+          <t>Không thiếu mapping</t>
         </is>
       </c>
     </row>
@@ -11188,32 +12068,32 @@
       </c>
       <c r="B17" s="37" t="inlineStr">
         <is>
+          <t>DataModel</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>Chi tiết field-level cho Fact/Dim</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>Traceability</t>
+        </is>
+      </c>
+      <c r="E17" s="23" t="inlineStr">
+        <is>
           <t>ModelRelationships</t>
         </is>
       </c>
-      <c r="C17" s="23" t="inlineStr">
-        <is>
-          <t>Hiểu cardinality/filter direction</t>
-        </is>
-      </c>
-      <c r="D17" s="23" t="inlineStr">
-        <is>
-          <t>DataModel</t>
-        </is>
-      </c>
-      <c r="E17" s="23" t="inlineStr">
-        <is>
-          <t>SourceMapping</t>
-        </is>
-      </c>
       <c r="F17" s="23" t="inlineStr">
         <is>
-          <t>Power BI Dev</t>
+          <t>Data Modeler</t>
         </is>
       </c>
       <c r="G17" s="23" t="inlineStr">
         <is>
-          <t>Tránh lỗi filter mơ hồ</t>
+          <t>Build model chính xác</t>
         </is>
       </c>
     </row>
@@ -11223,32 +12103,32 @@
       </c>
       <c r="B18" s="37" t="inlineStr">
         <is>
+          <t>ModelRelationships</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu cardinality/filter direction</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>DataModel</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="inlineStr">
+        <is>
           <t>SourceMapping</t>
         </is>
       </c>
-      <c r="C18" s="23" t="inlineStr">
-        <is>
-          <t>Map source field -&gt; semantic field + transform</t>
-        </is>
-      </c>
-      <c r="D18" s="23" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="E18" s="23" t="inlineStr">
-        <is>
-          <t>DAXLogic</t>
-        </is>
-      </c>
       <c r="F18" s="23" t="inlineStr">
         <is>
-          <t>ETL Dev</t>
+          <t>Power BI Dev</t>
         </is>
       </c>
       <c r="G18" s="23" t="inlineStr">
         <is>
-          <t>Triển khai ETL chuẩn</t>
+          <t>Tránh filter ambiguity</t>
         </is>
       </c>
     </row>
@@ -11258,32 +12138,32 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
+          <t>SourceMapping</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>Map source -&gt; semantic + transform</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="E19" s="23" t="inlineStr">
+        <is>
           <t>DAXLogic</t>
         </is>
       </c>
-      <c r="C19" s="23" t="inlineStr">
-        <is>
-          <t>Công thức DAX đầy đủ + test case</t>
-        </is>
-      </c>
-      <c r="D19" s="23" t="inlineStr">
-        <is>
-          <t>KPI + Mapping</t>
-        </is>
-      </c>
-      <c r="E19" s="23" t="inlineStr">
-        <is>
-          <t>BusinessRules</t>
-        </is>
-      </c>
       <c r="F19" s="23" t="inlineStr">
         <is>
-          <t>Power BI Dev</t>
+          <t>ETL Dev</t>
         </is>
       </c>
       <c r="G19" s="23" t="inlineStr">
         <is>
-          <t>Measure chạy đúng logic</t>
+          <t>Triển khai ETL chuẩn</t>
         </is>
       </c>
     </row>
@@ -11293,32 +12173,32 @@
       </c>
       <c r="B20" s="37" t="inlineStr">
         <is>
+          <t>DAXLogic</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>Công thức DAX đầy đủ + test case</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t>KPI + Mapping</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="inlineStr">
+        <is>
           <t>BusinessRules</t>
         </is>
       </c>
-      <c r="C20" s="23" t="inlineStr">
-        <is>
-          <t>Luật nghiệp vụ và ngoại lệ ngành xây dựng</t>
-        </is>
-      </c>
-      <c r="D20" s="23" t="inlineStr">
-        <is>
-          <t>DAX</t>
-        </is>
-      </c>
-      <c r="E20" s="23" t="inlineStr">
-        <is>
-          <t>RLS_Heatmap_v2</t>
-        </is>
-      </c>
       <c r="F20" s="23" t="inlineStr">
         <is>
-          <t>Business + QA</t>
+          <t>Power BI Dev</t>
         </is>
       </c>
       <c r="G20" s="23" t="inlineStr">
         <is>
-          <t>Bộ rule kiểm thử hoàn chỉnh</t>
+          <t>Measure chạy đúng logic</t>
         </is>
       </c>
     </row>
@@ -11328,32 +12208,32 @@
       </c>
       <c r="B21" s="37" t="inlineStr">
         <is>
+          <t>BusinessRules</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>Luật nghiệp vụ và ngoại lệ</t>
+        </is>
+      </c>
+      <c r="D21" s="23" t="inlineStr">
+        <is>
+          <t>DAX</t>
+        </is>
+      </c>
+      <c r="E21" s="23" t="inlineStr">
+        <is>
           <t>RLS_Heatmap_v2</t>
         </is>
       </c>
-      <c r="C21" s="23" t="inlineStr">
-        <is>
-          <t>Nhìn nhanh phạm vi role và access</t>
-        </is>
-      </c>
-      <c r="D21" s="23" t="inlineStr">
-        <is>
-          <t>BusinessRules</t>
-        </is>
-      </c>
-      <c r="E21" s="23" t="inlineStr">
-        <is>
-          <t>RLS</t>
-        </is>
-      </c>
       <c r="F21" s="23" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Business + QA</t>
         </is>
       </c>
       <c r="G21" s="23" t="inlineStr">
         <is>
-          <t>Xác nhận policy trước publish</t>
+          <t>Bộ rule kiểm thử hoàn chỉnh</t>
         </is>
       </c>
     </row>
@@ -11363,32 +12243,32 @@
       </c>
       <c r="B22" s="37" t="inlineStr">
         <is>
+          <t>RLS_Heatmap_v2</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
+          <t>Nhìn nhanh phạm vi role và access</t>
+        </is>
+      </c>
+      <c r="D22" s="23" t="inlineStr">
+        <is>
+          <t>BusinessRules</t>
+        </is>
+      </c>
+      <c r="E22" s="23" t="inlineStr">
+        <is>
           <t>RLS</t>
         </is>
       </c>
-      <c r="C22" s="23" t="inlineStr">
-        <is>
-          <t>DAX filter role-level cho Power BI Service</t>
-        </is>
-      </c>
-      <c r="D22" s="23" t="inlineStr">
-        <is>
-          <t>RLS Heatmap</t>
-        </is>
-      </c>
-      <c r="E22" s="23" t="inlineStr">
-        <is>
-          <t>Refresh_Monitor_v2</t>
-        </is>
-      </c>
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>Security + Admin</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="G22" s="23" t="inlineStr">
         <is>
-          <t>Thiết lập phân quyền chính thức</t>
+          <t>Xác nhận policy trước publish</t>
         </is>
       </c>
     </row>
@@ -11398,37 +12278,72 @@
       </c>
       <c r="B23" s="37" t="inlineStr">
         <is>
+          <t>RLS</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="inlineStr">
+        <is>
+          <t>DAX filter role-level trong service</t>
+        </is>
+      </c>
+      <c r="D23" s="23" t="inlineStr">
+        <is>
+          <t>RLS heatmap</t>
+        </is>
+      </c>
+      <c r="E23" s="23" t="inlineStr">
+        <is>
           <t>Refresh_Monitor_v2</t>
         </is>
       </c>
-      <c r="C23" s="23" t="inlineStr">
+      <c r="F23" s="23" t="inlineStr">
+        <is>
+          <t>Security + Admin</t>
+        </is>
+      </c>
+      <c r="G23" s="23" t="inlineStr">
+        <is>
+          <t>Thiết lập phân quyền chính thức</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="24" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" s="37" t="inlineStr">
+        <is>
+          <t>Refresh_Monitor_v2</t>
+        </is>
+      </c>
+      <c r="C24" s="23" t="inlineStr">
         <is>
           <t>Theo dõi vận hành refresh/DQ sau triển khai</t>
         </is>
       </c>
-      <c r="D23" s="23" t="inlineStr">
+      <c r="D24" s="23" t="inlineStr">
         <is>
           <t>All implementation</t>
         </is>
       </c>
-      <c r="E23" s="23" t="inlineStr">
+      <c r="E24" s="23" t="inlineStr">
         <is>
           <t>Runbook</t>
         </is>
       </c>
-      <c r="F23" s="23" t="inlineStr">
+      <c r="F24" s="23" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="G23" s="23" t="inlineStr">
+      <c r="G24" s="23" t="inlineStr">
         <is>
           <t>Sẵn sàng go-live monitoring</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:G23"/>
+  <autoFilter ref="A6:G24"/>
   <mergeCells count="2">
     <mergeCell ref="A3:G4"/>
     <mergeCell ref="A1:G2"/>
@@ -11451,12 +12366,452 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="85" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rule ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Phân hệ</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Luật nghiệp vụ chi tiết</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Điểm triển khai</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Xử lý ngoại lệ</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Data Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>BR-01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Mã vật tư phải map MaterialGroup; không map gán UNCLASSIFIED và alert 08:00 mỗi ngày.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>ETL SQL + Power Query</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Vẫn load nhưng loại khỏi KPI chiến lược.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>MDM Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>BR-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>NormQty lấy theo BOM approved mới nhất có EffectiveDate &lt;= ngày giao dịch.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>ETL SQL</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Không có BOM thì Overuse KPI trả BLANK và log DQ.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Engineering Control</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>BR-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ load dự án Status IN ('Active','Closing'); Closed giữ tối đa 24 tháng.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>ETL SQL</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Audit sâu dùng workspace archive.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>PMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>BR-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>ActualAmount loại bút toán reversal/cancelled theo trạng thái chứng từ.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ETL SQL</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Reversal đến sau cutoff ghi adjustment kỳ kế tiếp.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>BR-05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Quy đổi currency về VND theo tỷ giá cuối tháng; thiếu rate dùng nearest previous.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Power Query + SQL</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Thiếu rate &gt;7 ngày đánh critical.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Treasury</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>BR-06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Progress</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>DelayDays = max(0, ForecastFinishDate - PlannedFinishDate).</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>ETL SQL</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Forecast null dùng RevisedFinishDate.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Planning Office</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>BR-07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Progress</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Actual Progress % cap 100% để tránh outlier do baseline cập nhật trễ.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>DAX</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Record &gt;100% được log để PM xác nhận.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Planning Office</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>BR-08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Productivity Index chỉ tính khi LaborHours&gt;0 và ActualCompletedQty&gt;0.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>DAX</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Record không hợp lệ đưa vào trang Data Quality.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Contract Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>BR-09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>User chỉ xem dự án mapping trong SecurityUserProject và IsActive=1.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>RLS DAX</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>User không mapping sẽ không thấy dữ liệu.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>IT Security</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>BR-10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Khóa số liệu tháng vào T+3 18:00; sửa sau khóa cần approval ticket.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Process + SQL</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Lưu audit trail DataCorrectionLog.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>PMO + Data Governance</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>BR-11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Executive dashboard chỉ hiển thị Top 15 dự án theo Actual Cost để tối ưu hiệu năng.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Visual Filter</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Danh sách đầy đủ ở drillthrough.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>BI Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>BR-12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Đối soát KPI semantic vs source hằng ngày; sai lệch cho phép &lt;=0.5%.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>SQL Validation Job</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Lệch &gt;0.5% thì refresh fail + gửi alert.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Data Quality Team</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13565,7 +14920,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>v2.1 - Detail Design (Visual + Navigation Linked)</t>
+          <t>v2.2 - Detail Design (Visual + Navigation + Module Function Spec)</t>
         </is>
       </c>
     </row>
@@ -13605,7 +14960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13790,6 +15145,28 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>v2.2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Senior BI Solution Architect</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Bổ sung mô tả chức năng chi tiết cho từng module (must-have), thêm Module_Function_Spec_v2 và cập nhật luồng đọc.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Implement detailed DashboardCatalog spec for DD v2
Co-authored-by: nguyenpr9 <nguyenpr9@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Detail Design v2.xlsx
+++ b/Detail Design v2.xlsx
@@ -19,8 +19,8 @@
     <sheet name="Overview" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Modules" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Module_Function_Spec_v2" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="DashboardCatalog" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="DashboardLayoutSpec" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="DashboardLayoutSpec" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="DashboardCatalog" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="KPI" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="DataModel" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="ModelRelationships" sheetId="17" state="visible" r:id="rId17"/>
@@ -36,8 +36,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Overview'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Modules'!$A$1:$L$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Module_Function_Spec_v2'!$A$1:$J$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'DashboardCatalog'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'DashboardLayoutSpec'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'DashboardLayoutSpec'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'DashboardCatalog'!$A$1:$P$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'KPI'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'DataModel'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'ModelRelationships'!$A$1:$H$1</definedName>
@@ -1453,11 +1453,11 @@
           <t>NEW IN v2.2 - Module detail path</t>
         </is>
       </c>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="12" t="n"/>
-      <c r="E28" s="12" t="n"/>
-      <c r="F28" s="12" t="n"/>
-      <c r="G28" s="12" t="n"/>
+      <c r="C28" s="38" t="n"/>
+      <c r="D28" s="38" t="n"/>
+      <c r="E28" s="38" t="n"/>
+      <c r="F28" s="38" t="n"/>
+      <c r="G28" s="39" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="40" t="inlineStr">
@@ -1612,7 +1612,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="43" t="n"/>
       <c r="B9" s="43" t="n"/>
@@ -1631,7 +1630,11 @@
     </row>
     <row r="11">
       <c r="A11" s="43" t="n"/>
-      <c r="B11" s="44" t="n"/>
+      <c r="B11" s="44" t="inlineStr">
+        <is>
+          <t>#'00_ReadMe_Visual'!A1</t>
+        </is>
+      </c>
       <c r="C11" s="43" t="n"/>
       <c r="D11" s="43" t="n"/>
       <c r="E11" s="43" t="n"/>
@@ -1639,7 +1642,11 @@
     </row>
     <row r="12">
       <c r="A12" s="43" t="n"/>
-      <c r="B12" s="44" t="n"/>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t>#'ERD_Star_Visual_v2'!A1</t>
+        </is>
+      </c>
       <c r="C12" s="43" t="n"/>
       <c r="D12" s="43" t="n"/>
       <c r="E12" s="43" t="n"/>
@@ -1647,7 +1654,11 @@
     </row>
     <row r="13">
       <c r="A13" s="43" t="n"/>
-      <c r="B13" s="44" t="n"/>
+      <c r="B13" s="44" t="inlineStr">
+        <is>
+          <t>#'ETL_Swimlane_v2'!A1</t>
+        </is>
+      </c>
       <c r="C13" s="43" t="n"/>
       <c r="D13" s="43" t="n"/>
       <c r="E13" s="43" t="n"/>
@@ -1655,7 +1666,11 @@
     </row>
     <row r="14">
       <c r="A14" s="43" t="n"/>
-      <c r="B14" s="44" t="n"/>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t>#'Overview'!A1</t>
+        </is>
+      </c>
       <c r="C14" s="43" t="n"/>
       <c r="D14" s="43" t="n"/>
       <c r="E14" s="43" t="n"/>
@@ -1663,7 +1678,11 @@
     </row>
     <row r="15">
       <c r="A15" s="43" t="n"/>
-      <c r="B15" s="44" t="n"/>
+      <c r="B15" s="44" t="inlineStr">
+        <is>
+          <t>#'Modules'!A1</t>
+        </is>
+      </c>
       <c r="C15" s="43" t="n"/>
       <c r="D15" s="43" t="n"/>
       <c r="E15" s="43" t="n"/>
@@ -1671,7 +1690,11 @@
     </row>
     <row r="16">
       <c r="A16" s="43" t="n"/>
-      <c r="B16" s="44" t="n"/>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t>#'DashboardCatalog'!A1</t>
+        </is>
+      </c>
       <c r="C16" s="43" t="n"/>
       <c r="D16" s="43" t="n"/>
       <c r="E16" s="43" t="n"/>
@@ -1679,7 +1702,11 @@
     </row>
     <row r="17">
       <c r="A17" s="43" t="n"/>
-      <c r="B17" s="44" t="n"/>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t>#'DashboardLayoutSpec'!A1</t>
+        </is>
+      </c>
       <c r="C17" s="43" t="n"/>
       <c r="D17" s="43" t="n"/>
       <c r="E17" s="43" t="n"/>
@@ -1687,7 +1714,11 @@
     </row>
     <row r="18">
       <c r="A18" s="43" t="n"/>
-      <c r="B18" s="44" t="n"/>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t>#'KPI'!A1</t>
+        </is>
+      </c>
       <c r="C18" s="43" t="n"/>
       <c r="D18" s="43" t="n"/>
       <c r="E18" s="43" t="n"/>
@@ -1695,7 +1726,11 @@
     </row>
     <row r="19">
       <c r="A19" s="43" t="n"/>
-      <c r="B19" s="44" t="n"/>
+      <c r="B19" s="44" t="inlineStr">
+        <is>
+          <t>#'Traceability_Matrix_v2'!A1</t>
+        </is>
+      </c>
       <c r="C19" s="43" t="n"/>
       <c r="D19" s="43" t="n"/>
       <c r="E19" s="43" t="n"/>
@@ -1703,7 +1738,11 @@
     </row>
     <row r="20">
       <c r="A20" s="43" t="n"/>
-      <c r="B20" s="44" t="n"/>
+      <c r="B20" s="44" t="inlineStr">
+        <is>
+          <t>#'DataModel'!A1</t>
+        </is>
+      </c>
       <c r="C20" s="43" t="n"/>
       <c r="D20" s="43" t="n"/>
       <c r="E20" s="43" t="n"/>
@@ -1711,7 +1750,11 @@
     </row>
     <row r="21">
       <c r="A21" s="43" t="n"/>
-      <c r="B21" s="44" t="n"/>
+      <c r="B21" s="44" t="inlineStr">
+        <is>
+          <t>#'ModelRelationships'!A1</t>
+        </is>
+      </c>
       <c r="C21" s="43" t="n"/>
       <c r="D21" s="43" t="n"/>
       <c r="E21" s="43" t="n"/>
@@ -1719,7 +1762,11 @@
     </row>
     <row r="22">
       <c r="A22" s="43" t="n"/>
-      <c r="B22" s="44" t="n"/>
+      <c r="B22" s="44" t="inlineStr">
+        <is>
+          <t>#'SourceMapping'!A1</t>
+        </is>
+      </c>
       <c r="C22" s="43" t="n"/>
       <c r="D22" s="43" t="n"/>
       <c r="E22" s="43" t="n"/>
@@ -1727,7 +1774,11 @@
     </row>
     <row r="23">
       <c r="A23" s="43" t="n"/>
-      <c r="B23" s="44" t="n"/>
+      <c r="B23" s="44" t="inlineStr">
+        <is>
+          <t>#'DAXLogic'!A1</t>
+        </is>
+      </c>
       <c r="C23" s="43" t="n"/>
       <c r="D23" s="43" t="n"/>
       <c r="E23" s="43" t="n"/>
@@ -1735,7 +1786,11 @@
     </row>
     <row r="24">
       <c r="A24" s="43" t="n"/>
-      <c r="B24" s="44" t="n"/>
+      <c r="B24" s="44" t="inlineStr">
+        <is>
+          <t>#'BusinessRules'!A1</t>
+        </is>
+      </c>
       <c r="C24" s="43" t="n"/>
       <c r="D24" s="43" t="n"/>
       <c r="E24" s="43" t="n"/>
@@ -1743,7 +1798,11 @@
     </row>
     <row r="25">
       <c r="A25" s="43" t="n"/>
-      <c r="B25" s="44" t="n"/>
+      <c r="B25" s="44" t="inlineStr">
+        <is>
+          <t>#'RLS_Heatmap_v2'!A1</t>
+        </is>
+      </c>
       <c r="C25" s="43" t="n"/>
       <c r="D25" s="43" t="n"/>
       <c r="E25" s="43" t="n"/>
@@ -1751,7 +1810,11 @@
     </row>
     <row r="26">
       <c r="A26" s="43" t="n"/>
-      <c r="B26" s="44" t="n"/>
+      <c r="B26" s="44" t="inlineStr">
+        <is>
+          <t>#'RLS'!A1</t>
+        </is>
+      </c>
       <c r="C26" s="43" t="n"/>
       <c r="D26" s="43" t="n"/>
       <c r="E26" s="43" t="n"/>
@@ -1759,7 +1822,11 @@
     </row>
     <row r="27">
       <c r="A27" s="43" t="n"/>
-      <c r="B27" s="44" t="n"/>
+      <c r="B27" s="44" t="inlineStr">
+        <is>
+          <t>#'Refresh_Monitor_v2'!A1</t>
+        </is>
+      </c>
       <c r="C27" s="43" t="n"/>
       <c r="D27" s="43" t="n"/>
       <c r="E27" s="43" t="n"/>
@@ -1771,11 +1838,11 @@
           <t>NAVIGATION FROM OVERVIEW</t>
         </is>
       </c>
-      <c r="B29" s="1" t="n"/>
-      <c r="C29" s="1" t="n"/>
-      <c r="D29" s="1" t="n"/>
-      <c r="E29" s="1" t="n"/>
-      <c r="F29" s="1" t="n"/>
+      <c r="B29" s="38" t="n"/>
+      <c r="C29" s="38" t="n"/>
+      <c r="D29" s="38" t="n"/>
+      <c r="E29" s="38" t="n"/>
+      <c r="F29" s="39" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
@@ -3755,224 +3822,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="69" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="85" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="52" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Trang</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Mục tiêu</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Người dùng</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Layout tổng quan</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Mockup ASCII</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Insight hành động</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Executive Portfolio Overview</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Portfolio Summary</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Bức tranh tổng quan ngân sách + tiến độ + rủi ro ở cấp portfolio.</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>CEO, COO, PMO Director</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Row1 KPI x6; Row2-left column actual vs budget; Row2-right line cashflow; Row3 matrix overspend.</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>[KPI1][KPI2][KPI3][KPI4][KPI5][KPI6]
-[Actual vs Budget] [Cashflow]
-[Matrix Overspend]</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Ưu tiên dự án Variance% &gt; 10% và SPI &lt; 0.95.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Material Consumption Control</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Material Deep Dive</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Theo dõi tiêu thụ vật tư theo loại, dự án, nhà thầu, định mức.</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Project Manager, Site Engineer</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Top KPI x4; donut material mix; stacked column theo dự án; heatmap overuse; table drillthrough.</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>[KPI x4]
-[Donut] [Stacked Column] [Heatmap]
-[Transaction Table]</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Khoanh vùng contractor/work package gây overuse.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Cost vs Budget Deep Dive</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Cost Analysis</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Phân tích chênh lệch ngân sách theo category, contractor, timeline.</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Finance Controller, PM</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Top KPI; waterfall variance; bar theo category; treemap contractor; matrix drill path.</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>[KPI]
-[Waterfall] [Bar]
-[Treemap]
-[Matrix Drilldown]</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Xác định cost bucket cần cắt giảm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Progress &amp; Delay Risk</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Schedule Monitoring</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Giám sát tiến độ và dự báo trễ milestone.</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Planning Engineer, PM</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Top KPI; line planned vs actual; risk matrix; milestone table có conditional format.</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>[KPI]
-[Trend Line] [Risk Matrix]
-[Milestone Table]</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Ưu tiên hạng mục delay &gt; 7 ngày và risk score cao.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:G1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4702,6 +4551,624 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="54" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="70" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
+    <col width="70" customWidth="1" min="11" max="11"/>
+    <col width="67" customWidth="1" min="12" max="12"/>
+    <col width="70" customWidth="1" min="13" max="13"/>
+    <col width="70" customWidth="1" min="14" max="14"/>
+    <col width="55" customWidth="1" min="15" max="15"/>
+    <col width="48" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dashboard ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Dashboard / Page</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Business Objective</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Primary Persona</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Decision Supported</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Required Input Tables</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Mandatory Visual Contract</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Core Measures (DAX)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Default Filters &amp; Slicers</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Interaction / Drill Rules</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Layout Spec Reference</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>RLS &amp; Data Scope Notes</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Performance Target</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>UAT Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Owner / Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>DB-01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Executive Portfolio Overview / Portfolio Summary</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>M02 + M03</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Cung cấp bức tranh cấp điều hành về ngân sách, tiến độ và rủi ro portfolio.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>CEO, COO, PMO Director</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Quyết định phân bổ lại nguồn lực, ưu tiên dự án cần can thiệp.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>FactProjectCost, FactProgressTracking, DimProject, DimDate, DimCostCategory</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>6 KPI cards (Budget/Actual/Variance%/SPI/CPI/Risk Projects) + 1 clustered column + 1 line trend + 1 overspend matrix.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>[Budget Cost], [Actual Cost], [Budget Variance], [Budget Variance %], [SPI], [CPI], [Delay Risk Level]</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Default Year=Current Year; TopN 15 projects by Actual Cost; slicers: Region, Project Type, PM.</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Click bar project filters matrix + KPI context; matrix supports drill Project -&gt; Cost Category -&gt; Contractor.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>DashboardLayoutSpec: V01..V06</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>RLS theo ProjectKey. Role Site Engineer không được publish page này trong app role-based.</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>P95 query &lt; 4 giây; render first view &lt; 7 giây với 15 projects.</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>1) KPI khớp test set finance/progress
+2) Top overspend đúng sort
+3) Drilldown không mất filter context</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>PMO BI Team / Implemented (Phase-1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>DB-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Material Consumption Control / Material Deep Dive</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>M01</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Kiểm soát tiêu thụ vật tư và phát hiện vượt định mức theo contractor/work package.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Project Manager, Site Engineer, Procurement</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Quyết định điều chỉnh cấp phát vật tư, kiểm tra hao hụt bất thường, audit chứng từ.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>FactMaterialConsumption, DimMaterial, DimProject, DimContractor, DimWorkPackage, DimDate</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>4 KPI cards + donut material mix + stacked column by project + overuse heatmap + transaction table (drillthrough).</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>[Total Material Quantity], [Norm Quantity], [OverNorm Quantity], [Material Overuse %], [Return Rate]</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Default Date=Last 30 days; exclude UNCLASSIFIED on mix chart; optional slicer ContractorType.</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Click heatmap cell -&gt; drillthrough transaction detail (DocNo level); sync slicer across page visuals.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>DashboardLayoutSpec: V01..V06 (Material Deep Dive)</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>RLS: ProjectManager/SiteEngineer theo project mapping; ContractorViewer chỉ thấy own CompanyCode.</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>P95 query &lt; 4 giây; drillthrough detail page &lt; 6 giây (90-day window).</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>1) Overuse% = OverNorm/Norm đúng theo test TC-KPI-002
+2) Drillthrough mở đúng SourceDocNo
+3) Filter đồng bộ các visual</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Procurement BI Squad / Implemented (Phase-1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>DB-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Cost vs Budget Deep Dive / Cost Analysis</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>M03</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Phân rã nguyên nhân chênh lệch ngân sách theo category, contractor và timeline.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Finance Controller, PM, PMO</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Quyết định cắt giảm chi phí, xử lý nhóm chi vượt mức và đánh giá tác động change order.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>FactProjectCost, DimCostCategory, DimContractor, DimProject, DimDate</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>4 KPI cards + waterfall variance bridge + bar variance by category + treemap contractor + matrix drill path.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>[Budget Cost], [Actual Cost], [Budget Variance], [Budget Variance %], [ChangeOrder Impact]</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Default Year=current; visual filter [Budget Variance %] &gt; 0 cho bảng overspend; slicers: Region, CostType.</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Select waterfall step filters matrix; matrix drill path Project -&gt; Category -&gt; Contractor; export summary only.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>DashboardLayoutSpec: V01..V04 (Cost Analysis)</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>RLS theo project; category Contingency không áp dụng cảnh báo màu vượt chi phí.</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>P95 query &lt; 4 giây với max 24 tháng dữ liệu; matrix expand level-3 &lt; 6 giây.</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>1) Variance waterfall tổng bằng KPI variance
+2) Category top-N đúng sort
+3) Cảnh báo 5/10% đúng màu</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Finance BI Analyst / Implemented (Phase-1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>DB-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Progress &amp; Delay Risk / Schedule Monitoring</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>M02</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi tiến độ thực tế vs kế hoạch và đánh giá rủi ro trễ milestone.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Planning Engineer, PM</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Quyết định ưu tiên gói công việc cần bù tiến độ và xử lý rủi ro cao.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>FactProgressTracking, DimWorkPackage, DimProject, DimDate, DimContractor</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>4 KPI cards + planned/actual trend line + risk matrix + milestone warning table.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>[Planned Progress %], [Actual Progress %], [Delay Days], [SPI], [Delay Risk Level]</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Default Last 26 weeks; milestone table filter DelayDays &gt;= 3; slicers: Region, Phase, Contractor.</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Select risk bubble filters milestone table; drill Project -&gt; Phase -&gt; WorkPackage from table.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>DashboardLayoutSpec: V01..V03 (Schedule Monitoring)</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>RLS theo project; SiteEngineer truy cập page này, không truy cập cost pages.</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>P95 query &lt; 4 giây; risk matrix interaction &lt; 2 giây cho selection event.</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>1) Planned/Actual trend khớp source
+2) DelayDays âm được ép 0
+3) Risk level rule High/Medium/Low đúng biên</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>Planning BI Analyst / Implemented (Phase-1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>DB-05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Scorecard / Contractor Benchmark</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>M04</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Đánh giá hiệu suất nhà thầu theo productivity, SLA và mức độ tuân thủ.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Contract Manager, PMO</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Quyết định lựa chọn nhà thầu cho giai đoạn tiếp theo và kế hoạch cải thiện SLA.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>DimContractor, FactProgressTracking, FactMaterialConsumption, DeliveryPerformance</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>KPI tier cards + ranking table + SLA trend + benchmark matrix (planned).</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>[Contractor Productivity Index], [On-time Delivery %], [SLA Violation Count]</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Default last 3 months; slicers: ContractorType, Region, Project.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Drill contractor -&gt; project -&gt; work package; tooltip hiển thị SLA detail.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Layout pending (next sprint) - placeholder in DashboardLayoutSpec</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>ContractorViewer chỉ nhìn own company; internal roles có đầy đủ benchmark cross-contractor.</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>P95 query &lt; 5 giây sau khi triển khai page chuyên biệt.</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>1) Ranking stable theo weighted score
+2) External role không nhìn cross-company benchmark</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>Contract BI Product Owner / Planned (Sprint+2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>DB-06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance &amp; Billing Tracker / Acceptance to Payment</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>M05</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi vòng đời nghiệm thu -&gt; thanh toán và phát hiện hồ sơ quá hạn SLA.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>QS, Site Engineer, Finance Ops</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Quyết định đẩy nhanh hồ sơ pending và giảm tồn đọng thanh toán.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>AcceptanceMinutes, BillingProgress, PaymentCertificate, FactProgressTracking, DimDate</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>KPI accepted qty/pending amount + workflow funnel + pending list + delay alert table (planned).</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>[Accepted Qty], [Pending Billing Amount], [Payment Delay Days], [Billing SLA Breach %]</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Default current month + previous month; slicers: Project, Phase, BillingStatus.</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Click funnel status filters pending list; drill to certificate/document detail.</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Layout pending (next sprint) - placeholder in DashboardLayoutSpec</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>RLS theo project + role; ContractorViewer không truy cập billing amount chi tiết công ty nội bộ.</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>P95 query &lt; 5 giây với data window 12 tháng.</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>1) Pending amount đối soát AP
+2) Delay alert đúng SLA rule
+3) Drill tới chứng từ thanh toán chính xác</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>Finance Ops BI / Planned (Sprint+3)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11637,21 +12104,21 @@
           <t>DETAIL DESIGN - RECOMMENDED READING PATH (UPDATED WITH MODULE FUNCTION SPEC)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
+      <c r="B1" s="29" t="n"/>
+      <c r="C1" s="29" t="n"/>
+      <c r="D1" s="29" t="n"/>
+      <c r="E1" s="29" t="n"/>
+      <c r="F1" s="29" t="n"/>
+      <c r="G1" s="30" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n"/>
-      <c r="B2" s="1" t="n"/>
-      <c r="C2" s="1" t="n"/>
-      <c r="D2" s="1" t="n"/>
-      <c r="E2" s="1" t="n"/>
-      <c r="F2" s="1" t="n"/>
-      <c r="G2" s="1" t="n"/>
+      <c r="A2" s="31" t="n"/>
+      <c r="B2" s="32" t="n"/>
+      <c r="C2" s="32" t="n"/>
+      <c r="D2" s="32" t="n"/>
+      <c r="E2" s="32" t="n"/>
+      <c r="F2" s="32" t="n"/>
+      <c r="G2" s="33" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="40" t="inlineStr">
@@ -11659,21 +12126,21 @@
           <t>Đọc theo thứ tự. Cột "Liên kết sheet" có hyperlink. Bổ sung bước Module_Function_Spec_v2 để dev biết rõ từng module cần làm gì.</t>
         </is>
       </c>
-      <c r="B3" s="40" t="n"/>
-      <c r="C3" s="40" t="n"/>
-      <c r="D3" s="40" t="n"/>
-      <c r="E3" s="40" t="n"/>
-      <c r="F3" s="40" t="n"/>
-      <c r="G3" s="40" t="n"/>
+      <c r="B3" s="29" t="n"/>
+      <c r="C3" s="29" t="n"/>
+      <c r="D3" s="29" t="n"/>
+      <c r="E3" s="29" t="n"/>
+      <c r="F3" s="29" t="n"/>
+      <c r="G3" s="30" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="40" t="n"/>
-      <c r="B4" s="40" t="n"/>
-      <c r="C4" s="40" t="n"/>
-      <c r="D4" s="40" t="n"/>
-      <c r="E4" s="40" t="n"/>
-      <c r="F4" s="40" t="n"/>
-      <c r="G4" s="40" t="n"/>
+      <c r="A4" s="31" t="n"/>
+      <c r="B4" s="32" t="n"/>
+      <c r="C4" s="32" t="n"/>
+      <c r="D4" s="32" t="n"/>
+      <c r="E4" s="32" t="n"/>
+      <c r="F4" s="32" t="n"/>
+      <c r="G4" s="33" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -14920,7 +15387,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>v2.2 - Detail Design (Visual + Navigation + Module Function Spec)</t>
+          <t>v2.3 - Detail Design (DashboardCatalog implement-ready)</t>
         </is>
       </c>
     </row>
@@ -14960,7 +15427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15167,6 +15634,28 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>v2.3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Senior BI Solution Architect</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Nâng cấp DashboardCatalog lên mức implement: bổ sung visual contract, measure set, filter/interactions, UAT criteria và target hiệu năng.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Complete DashboardLayoutSpec for DB-05 and DB-06
Co-authored-by: nguyenpr9 <nguyenpr9@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Detail Design v2.xlsx
+++ b/Detail Design v2.xlsx
@@ -3822,21 +3822,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="68" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="33" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4546,6 +4546,762 @@
       <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Milestone cảnh báo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Scorecard</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Benchmark</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>CS01</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>[Contractor Productivity Index]</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Last 3 months</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Cross-highlight all visuals</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>KPI năng suất nhà thầu</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Scorecard</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Benchmark</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>CS02</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>[On-time Delivery %]</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Last 3 months</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Cross-highlight all visuals</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>KPI đúng hạn giao vật tư</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Scorecard</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Benchmark</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>CS03</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>[SLA Violation Count]</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Last 3 months</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Cross-highlight all visuals</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>KPI vi phạm SLA</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Scorecard</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Benchmark</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>CS04</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Axis:Contractor; Value:[Contractor Productivity Index]</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>TopN15 contractors</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Select contractor filters matrix + trend</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Xếp hạng nhà thầu theo năng suất</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Scorecard</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Benchmark</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>CS05</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>680</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Axis:Month; Values:[On-time Delivery %],[SLA Violation Count]</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Last 12 months</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Select month filters ranking + detail</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Xu hướng SLA theo thời gian</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Scorecard</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Benchmark</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>CS06</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Matrix</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>940</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Rows:Contractor-&gt;Project; Values:Productivity,On-time%,SLA Violations</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>ContractorType slicer</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Drill contractor -&gt; project</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Benchmark đa chỉ số</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Scorecard</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Contractor Benchmark</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>CS07</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>980</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>340</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Contractor,Project,WorkPackage,IssueType,IssueDate,Owner</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>SLA Violation Count &gt; 0</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Drillthrough to contractor detail</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Danh sách vi phạm chi tiết</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance &amp; Billing Tracker</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance to Payment</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>AB01</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>[Accepted Qty]</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Current + previous month</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Cross-highlight all visuals</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>KPI khối lượng nghiệm thu</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance &amp; Billing Tracker</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance to Payment</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>AB02</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>[Pending Billing Amount]</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Current + previous month</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Cross-highlight all visuals</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>KPI tồn đọng thanh toán</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance &amp; Billing Tracker</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance to Payment</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>AB03</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>[Payment Delay Days]</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Current + previous month</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Cross-highlight all visuals</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>KPI trễ thanh toán</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance &amp; Billing Tracker</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance to Payment</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>AB04</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Funnel</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>520</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Stage:BillingStatus; Value:DocumentCount</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Status in Pending/Approved/Paid</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Select stage filters pending list</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Workflow hồ sơ thanh toán</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance &amp; Billing Tracker</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance to Payment</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>AB05</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>560</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>760</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Axis:Project; Value:[Pending Billing Amount]</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>TopN15 by pending amount</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Select project filters tables</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Công trình tồn đọng cao</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance &amp; Billing Tracker</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance to Payment</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>AB06</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>940</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>DocNo,Project,Phase,AcceptedQty,BillingAmount,Status,DueDate</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Status &lt;&gt; Paid</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Drillthrough to certificate/document</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Danh sách hồ sơ pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance &amp; Billing Tracker</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance to Payment</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>AB07</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>980</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>340</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>DocNo,Project,DelayDays,Owner,ActionRequired</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>DelayDays &gt; 0</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Conditional color + alert action</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Danh sách quá hạn SLA</t>
         </is>
       </c>
     </row>
@@ -5038,7 +5794,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>KPI tier cards + ranking table + SLA trend + benchmark matrix (planned).</t>
+          <t>3 KPI tier cards + contractor ranking bar + SLA trend line + benchmark matrix + detail drill table.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -5058,7 +5814,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Layout pending (next sprint) - placeholder in DashboardLayoutSpec</t>
+          <t>DashboardLayoutSpec: CS01..CS07 (Contractor Benchmark)</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -5079,7 +5835,7 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>Contract BI Product Owner / Planned (Sprint+2)</t>
+          <t>Contract BI Product Owner / Design Ready (Sprint+2)</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5877,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>KPI accepted qty/pending amount + workflow funnel + pending list + delay alert table (planned).</t>
+          <t>3 KPI cards + billing workflow funnel + pending list table + delay alert table + document drillthrough.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -5141,7 +5897,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Layout pending (next sprint) - placeholder in DashboardLayoutSpec</t>
+          <t>DashboardLayoutSpec: AB01..AB07 (Acceptance to Payment)</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -5163,7 +5919,7 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>Finance Ops BI / Planned (Sprint+3)</t>
+          <t>Finance Ops BI / Design Ready (Sprint+3)</t>
         </is>
       </c>
     </row>
@@ -15387,7 +16143,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>v2.3 - Detail Design (DashboardCatalog implement-ready)</t>
+          <t>v2.4 - Detail Design (DashboardCatalog + LayoutSpec aligned)</t>
         </is>
       </c>
     </row>
@@ -15427,7 +16183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15656,6 +16412,28 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>v2.4</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Senior BI Solution Architect</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Hoàn thiện đồng bộ DashboardCatalog và DashboardLayoutSpec cho DB-05/DB-06 (design ready for implementation).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>